<commit_message>
compatible with double title rows in xls/xlas
</commit_message>
<xml_diff>
--- a/robustness/data/_robustness/all_claims.xlsx
+++ b/robustness/data/_robustness/all_claims.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\mason\mygpu\llm-robustness\llm-benchmarking-robustness\robustness\data\_robustness\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{984C0B7C-3B68-43D4-8A5F-966BFCAC38C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{702293D1-82ED-4C6A-A6E9-AB43FB149569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-6705" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3464,9 +3464,6 @@
     <t>Organizing the global value chain</t>
   </si>
   <si>
-    <t>Antràs_Econometrica_2013_a2Yx</t>
-  </si>
-  <si>
     <t>We uncover a positive ... relationship between each of the measures of downstreamness and the intrafirm import share in a given sector, with this relationship emerging only for high values of the demand elasticity faced by buyer industries (p. 2132.)</t>
   </si>
   <si>
@@ -3834,6 +3831,9 @@
   </si>
   <si>
     <t>Bingham Powell_CompPolitStu_2009_0PZl</t>
+  </si>
+  <si>
+    <t>AntrAs_Econometrica_2013_a2Yx</t>
   </si>
 </sst>
 </file>
@@ -9369,7 +9369,7 @@
         <v>950</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>107</v>
@@ -9587,7 +9587,7 @@
         <v>985</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>986</v>
+        <v>1078</v>
       </c>
       <c r="C91" s="4" t="s">
         <v>32</v>
@@ -9605,19 +9605,19 @@
         <v>438</v>
       </c>
       <c r="H91" s="8" t="s">
+        <v>986</v>
+      </c>
+      <c r="I91" s="9" t="s">
         <v>987</v>
       </c>
-      <c r="I91" s="9" t="s">
+      <c r="J91" s="4" t="s">
         <v>988</v>
       </c>
-      <c r="J91" s="4" t="s">
+      <c r="K91" s="4" t="s">
         <v>989</v>
       </c>
-      <c r="K91" s="4" t="s">
+      <c r="L91" s="23" t="s">
         <v>990</v>
-      </c>
-      <c r="L91" s="23" t="s">
-        <v>991</v>
       </c>
       <c r="M91" s="4"/>
       <c r="N91" s="7" t="s">
@@ -9635,15 +9635,15 @@
       </c>
       <c r="S91" s="7"/>
       <c r="T91" s="11" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
     </row>
     <row r="92" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
+        <v>992</v>
+      </c>
+      <c r="B92" s="4" t="s">
         <v>993</v>
-      </c>
-      <c r="B92" s="4" t="s">
-        <v>994</v>
       </c>
       <c r="C92" s="4" t="s">
         <v>107</v>
@@ -9661,19 +9661,19 @@
         <v>142</v>
       </c>
       <c r="H92" s="8" t="s">
+        <v>994</v>
+      </c>
+      <c r="I92" s="9" t="s">
         <v>995</v>
       </c>
-      <c r="I92" s="9" t="s">
+      <c r="J92" s="4" t="s">
         <v>996</v>
       </c>
-      <c r="J92" s="4" t="s">
+      <c r="K92" s="4" t="s">
         <v>997</v>
       </c>
-      <c r="K92" s="4" t="s">
+      <c r="L92" s="11" t="s">
         <v>998</v>
-      </c>
-      <c r="L92" s="11" t="s">
-        <v>999</v>
       </c>
       <c r="M92" s="4"/>
       <c r="N92" s="7" t="s">
@@ -9691,15 +9691,15 @@
       </c>
       <c r="S92" s="7"/>
       <c r="T92" s="11" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
     <row r="93" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B93" s="4" t="s">
         <v>1001</v>
-      </c>
-      <c r="B93" s="4" t="s">
-        <v>1002</v>
       </c>
       <c r="C93" s="4" t="s">
         <v>32</v>
@@ -9717,19 +9717,19 @@
         <v>142</v>
       </c>
       <c r="H93" s="33" t="s">
+        <v>1002</v>
+      </c>
+      <c r="I93" s="9" t="s">
         <v>1003</v>
       </c>
-      <c r="I93" s="9" t="s">
+      <c r="J93" s="7" t="s">
         <v>1004</v>
       </c>
-      <c r="J93" s="7" t="s">
+      <c r="K93" s="7" t="s">
         <v>1005</v>
       </c>
-      <c r="K93" s="7" t="s">
+      <c r="L93" s="43" t="s">
         <v>1006</v>
-      </c>
-      <c r="L93" s="43" t="s">
-        <v>1007</v>
       </c>
       <c r="M93" s="7"/>
       <c r="N93" s="7" t="s">
@@ -9743,19 +9743,19 @@
       </c>
       <c r="Q93" s="7"/>
       <c r="R93" s="7" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="S93" s="7"/>
       <c r="T93" s="43" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="94" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="7" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B94" s="7" t="s">
         <v>1010</v>
-      </c>
-      <c r="B94" s="7" t="s">
-        <v>1011</v>
       </c>
       <c r="C94" s="7" t="s">
         <v>576</v>
@@ -9773,19 +9773,19 @@
         <v>108</v>
       </c>
       <c r="H94" s="33" t="s">
+        <v>1011</v>
+      </c>
+      <c r="I94" s="9" t="s">
         <v>1012</v>
       </c>
-      <c r="I94" s="9" t="s">
+      <c r="J94" s="7" t="s">
         <v>1013</v>
       </c>
-      <c r="J94" s="7" t="s">
+      <c r="K94" s="7" t="s">
         <v>1014</v>
       </c>
-      <c r="K94" s="7" t="s">
+      <c r="L94" s="25" t="s">
         <v>1015</v>
-      </c>
-      <c r="L94" s="25" t="s">
-        <v>1016</v>
       </c>
       <c r="M94" s="7"/>
       <c r="N94" s="7" t="s">
@@ -9803,15 +9803,15 @@
       </c>
       <c r="S94" s="7"/>
       <c r="T94" s="43" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="95" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="7" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B95" s="7" t="s">
         <v>1018</v>
-      </c>
-      <c r="B95" s="7" t="s">
-        <v>1019</v>
       </c>
       <c r="C95" s="7" t="s">
         <v>576</v>
@@ -9829,19 +9829,19 @@
         <v>142</v>
       </c>
       <c r="H95" s="33" t="s">
+        <v>1019</v>
+      </c>
+      <c r="I95" s="9" t="s">
         <v>1020</v>
       </c>
-      <c r="I95" s="9" t="s">
+      <c r="J95" s="7" t="s">
         <v>1021</v>
       </c>
-      <c r="J95" s="7" t="s">
+      <c r="K95" s="7" t="s">
         <v>1022</v>
       </c>
-      <c r="K95" s="7" t="s">
+      <c r="L95" s="23" t="s">
         <v>1023</v>
-      </c>
-      <c r="L95" s="23" t="s">
-        <v>1024</v>
       </c>
       <c r="M95" s="7"/>
       <c r="N95" s="4" t="s">
@@ -9859,15 +9859,15 @@
       </c>
       <c r="S95" s="7"/>
       <c r="T95" s="43" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="96" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="7" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B96" s="7" t="s">
         <v>1026</v>
-      </c>
-      <c r="B96" s="7" t="s">
-        <v>1027</v>
       </c>
       <c r="C96" s="7" t="s">
         <v>576</v>
@@ -9885,19 +9885,19 @@
         <v>142</v>
       </c>
       <c r="H96" s="33" t="s">
+        <v>1027</v>
+      </c>
+      <c r="I96" s="9" t="s">
         <v>1028</v>
       </c>
-      <c r="I96" s="9" t="s">
+      <c r="J96" s="7" t="s">
         <v>1029</v>
       </c>
-      <c r="J96" s="7" t="s">
+      <c r="K96" s="7" t="s">
         <v>1030</v>
       </c>
-      <c r="K96" s="7" t="s">
+      <c r="L96" s="26" t="s">
         <v>1031</v>
-      </c>
-      <c r="L96" s="26" t="s">
-        <v>1032</v>
       </c>
       <c r="M96" s="4"/>
       <c r="N96" s="7"/>
@@ -9907,15 +9907,15 @@
       <c r="R96" s="7"/>
       <c r="S96" s="7"/>
       <c r="T96" s="43" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="97" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="7" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B97" s="7" t="s">
         <v>1034</v>
-      </c>
-      <c r="B97" s="7" t="s">
-        <v>1035</v>
       </c>
       <c r="C97" s="7" t="s">
         <v>107</v>
@@ -9933,19 +9933,19 @@
         <v>142</v>
       </c>
       <c r="H97" s="33" t="s">
+        <v>1035</v>
+      </c>
+      <c r="I97" s="9" t="s">
         <v>1036</v>
       </c>
-      <c r="I97" s="9" t="s">
+      <c r="J97" s="7" t="s">
         <v>1037</v>
       </c>
-      <c r="J97" s="7" t="s">
+      <c r="K97" s="7" t="s">
         <v>1038</v>
       </c>
-      <c r="K97" s="7" t="s">
+      <c r="L97" s="43" t="s">
         <v>1039</v>
-      </c>
-      <c r="L97" s="43" t="s">
-        <v>1040</v>
       </c>
       <c r="M97" s="7"/>
       <c r="N97" s="4" t="s">
@@ -9955,23 +9955,23 @@
         <v>50.110030000000002</v>
       </c>
       <c r="P97" s="44" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="Q97" s="7"/>
       <c r="R97" s="44" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="S97" s="7"/>
       <c r="T97" s="43" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="98" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="7" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B98" s="7" t="s">
         <v>1044</v>
-      </c>
-      <c r="B98" s="7" t="s">
-        <v>1045</v>
       </c>
       <c r="C98" s="7" t="s">
         <v>576</v>
@@ -9989,19 +9989,19 @@
         <v>36</v>
       </c>
       <c r="H98" s="33" t="s">
+        <v>1045</v>
+      </c>
+      <c r="I98" s="9" t="s">
         <v>1046</v>
       </c>
-      <c r="I98" s="9" t="s">
+      <c r="J98" s="7" t="s">
         <v>1047</v>
       </c>
-      <c r="J98" s="7" t="s">
+      <c r="K98" s="7" t="s">
         <v>1048</v>
       </c>
-      <c r="K98" s="7" t="s">
+      <c r="L98" s="25" t="s">
         <v>1049</v>
-      </c>
-      <c r="L98" s="25" t="s">
-        <v>1050</v>
       </c>
       <c r="M98" s="7"/>
       <c r="N98" s="7" t="s">
@@ -10019,15 +10019,15 @@
       </c>
       <c r="S98" s="7"/>
       <c r="T98" s="43" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="99" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="7" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B99" s="7" t="s">
         <v>1052</v>
-      </c>
-      <c r="B99" s="7" t="s">
-        <v>1053</v>
       </c>
       <c r="C99" s="7" t="s">
         <v>141</v>
@@ -10045,19 +10045,19 @@
         <v>142</v>
       </c>
       <c r="H99" s="33" t="s">
+        <v>1053</v>
+      </c>
+      <c r="I99" s="9" t="s">
         <v>1054</v>
       </c>
-      <c r="I99" s="9" t="s">
+      <c r="J99" s="7" t="s">
         <v>1055</v>
       </c>
-      <c r="J99" s="7" t="s">
+      <c r="K99" s="7" t="s">
         <v>1056</v>
       </c>
-      <c r="K99" s="7" t="s">
+      <c r="L99" s="26" t="s">
         <v>1057</v>
-      </c>
-      <c r="L99" s="26" t="s">
-        <v>1058</v>
       </c>
       <c r="M99" s="7"/>
       <c r="N99" s="7" t="s">
@@ -10073,18 +10073,18 @@
       <c r="R99" s="7"/>
       <c r="S99" s="7"/>
       <c r="T99" s="43" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="100" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="7" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B100" s="7" t="s">
         <v>1060</v>
       </c>
-      <c r="B100" s="7" t="s">
+      <c r="C100" s="7" t="s">
         <v>1061</v>
-      </c>
-      <c r="C100" s="7" t="s">
-        <v>1062</v>
       </c>
       <c r="D100" s="4" t="s">
         <v>672</v>
@@ -10099,19 +10099,19 @@
         <v>36</v>
       </c>
       <c r="H100" s="33" t="s">
+        <v>1062</v>
+      </c>
+      <c r="I100" s="9" t="s">
         <v>1063</v>
       </c>
-      <c r="I100" s="9" t="s">
+      <c r="J100" s="7" t="s">
         <v>1064</v>
       </c>
-      <c r="J100" s="7" t="s">
+      <c r="K100" s="7" t="s">
         <v>1065</v>
       </c>
-      <c r="K100" s="7" t="s">
+      <c r="L100" s="23" t="s">
         <v>1066</v>
-      </c>
-      <c r="L100" s="23" t="s">
-        <v>1067</v>
       </c>
       <c r="M100" s="7"/>
       <c r="N100" s="7" t="s">
@@ -10123,19 +10123,19 @@
       <c r="P100" s="7"/>
       <c r="Q100" s="7"/>
       <c r="R100" s="4" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="S100" s="7"/>
       <c r="T100" s="23" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="101" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="7" t="s">
+        <v>1069</v>
+      </c>
+      <c r="B101" s="7" t="s">
         <v>1070</v>
-      </c>
-      <c r="B101" s="7" t="s">
-        <v>1071</v>
       </c>
       <c r="C101" s="7" t="s">
         <v>141</v>
@@ -10153,19 +10153,19 @@
         <v>142</v>
       </c>
       <c r="H101" s="45" t="s">
+        <v>1071</v>
+      </c>
+      <c r="I101" s="9" t="s">
         <v>1072</v>
       </c>
-      <c r="I101" s="9" t="s">
+      <c r="J101" s="7" t="s">
         <v>1073</v>
       </c>
-      <c r="J101" s="7" t="s">
+      <c r="K101" s="7" t="s">
         <v>1074</v>
       </c>
-      <c r="K101" s="7" t="s">
+      <c r="L101" s="23" t="s">
         <v>1075</v>
-      </c>
-      <c r="L101" s="23" t="s">
-        <v>1076</v>
       </c>
       <c r="M101" s="7"/>
       <c r="N101" s="7" t="s">
@@ -10183,7 +10183,7 @@
       </c>
       <c r="S101" s="7"/>
       <c r="T101" s="23" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="102" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>